<commit_message>
fix(resultados): reporta 8 instancias en vez de 36 en los Excel por grupo
count_instances() contaba los 36 archivos de data/evolution, pero el
experimento limita la evolución a las primeras 8 con
-p experiment.max.instances=8 (run_experiment.sh). Ahora lee ese
parámetro y reporta el número que realmente usa el protocolo.

Se regeneran los 6 Excel por grupo: cambian solo las 4 celdas de texto
afectadas (hoja Configuración filas 19 y 33, nota de la hoja
Estadísticas Promedio y Mejor). Los datos numéricos y la información de
la máquina donde corrió el experimento quedan idénticos. Se corrige
también la nota del árbol de carpetas en GUIA_EXPERIMENTO_COMPLETA.md.
</commit_message>
<xml_diff>
--- a/RESULTADOS_EXPERIMENTO_GRUPO0.xlsx
+++ b/RESULTADOS_EXPERIMENTO_GRUPO0.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Configuración" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen General" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Baseline por Instancia" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Estadísticas por Ejecución" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Best Fitness por Ejecución" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Estadísticas Promedio y Mejor" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen General" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline por Instancia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estadísticas por Ejecución" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Fitness por Ejecución" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estadísticas Promedio y Mejor" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -628,12 +628,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>36 instancias</t>
+          <t>8 instancias</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>(Cada individuo se evalúa con todas las instancias)</t>
+          <t>(Las primeras N de data/evolution según experiment.max.instances; cada individuo se evalúa con todas ellas)</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>• Cada individuo se evalúa con 36 instancias de prueba</t>
+          <t>• Cada individuo se evalúa con 8 instancias de prueba</t>
         </is>
       </c>
     </row>
@@ -10856,7 +10856,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>NOTA IMPORTANTE: AvgERP = Error Relativo Promedio (ERP) de TODA la población en esa generación. BestERP = Error Relativo Promedio (ERP) del MEJOR individuo de esa generación. Cada individuo se evalúa con 36 instancias de prueba. El ERP se calcula como: promedio de |óptimo - solución| / óptimo sobre todas las instancias.</t>
+          <t>NOTA IMPORTANTE: AvgERP = Error Relativo Promedio (ERP) de TODA la población en esa generación. BestERP = Error Relativo Promedio (ERP) del MEJOR individuo de esa generación. Cada individuo se evalúa con 8 instancias de prueba. El ERP se calcula como: promedio de |óptimo - solución| / óptimo sobre todas las instancias.</t>
         </is>
       </c>
     </row>

</xml_diff>